<commit_message>
Add cost and price columns to rank product orders
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016GtZZioynu6BNNHeRc885e
</commit_message>
<xml_diff>
--- a/rank_product_orders.xlsx
+++ b/rank_product_orders.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ランク別一覧" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,23 +15,34 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ランク未設定の店舗" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
       <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <sz val="6"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -63,7 +73,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -426,17 +436,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="3" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -480,6 +488,21 @@
           <t>合計</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>PC原価</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>店原価</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>店売価</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -510,6 +533,15 @@
       <c r="H2" s="3" t="n">
         <v>384.0333333333334</v>
       </c>
+      <c r="I2" s="3" t="n">
+        <v>110.01</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>150.7</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -540,6 +572,15 @@
       <c r="H3" s="3" t="n">
         <v>152.2666666666667</v>
       </c>
+      <c r="I3" s="3" t="n">
+        <v>207.92</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>284.82</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>429</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -570,6 +611,15 @@
       <c r="H4" s="3" t="n">
         <v>175.0333333333333</v>
       </c>
+      <c r="I4" s="3" t="n">
+        <v>134.34</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>184.03</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -600,6 +650,15 @@
       <c r="H5" s="3" t="n">
         <v>67.86666666666666</v>
       </c>
+      <c r="I5" s="3" t="n">
+        <v>166.68</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>225.55</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>375</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -630,6 +689,15 @@
       <c r="H6" s="3" t="n">
         <v>189.3666666666667</v>
       </c>
+      <c r="I6" s="3" t="n">
+        <v>86.09</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>117.89</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -660,6 +728,15 @@
       <c r="H7" s="3" t="n">
         <v>588.3666666666667</v>
       </c>
+      <c r="I7" s="3" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>94.97</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -690,6 +767,15 @@
       <c r="H8" s="3" t="n">
         <v>97.59999999999999</v>
       </c>
+      <c r="I8" s="3" t="n">
+        <v>130.32</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>177.54</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -720,6 +806,15 @@
       <c r="H9" s="3" t="n">
         <v>171.5333333333333</v>
       </c>
+      <c r="I9" s="3" t="n">
+        <v>158.83</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>217.58</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -750,6 +845,15 @@
       <c r="H10" s="3" t="n">
         <v>664.4</v>
       </c>
+      <c r="I10" s="3" t="n">
+        <v>100.98</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>136.14</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -780,6 +884,15 @@
       <c r="H11" s="3" t="n">
         <v>384.3666666666667</v>
       </c>
+      <c r="I11" s="3" t="n">
+        <v>91.98</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>125.06</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -810,635 +923,365 @@
       <c r="H12" s="3" t="n">
         <v>211.3333333333333</v>
       </c>
+      <c r="I12" s="3" t="n">
+        <v>88.78</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>121.62</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2543875000000</t>
+          <t>2553097000000</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ふわもちホテルロール８個入</t>
+          <t>バナナのふんわりロール２</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>309.7333333333333</v>
+        <v>272.1333333333333</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>43.93333333333333</v>
+        <v>65.43333333333334</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>6.7</v>
+        <v>14.6</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>26.9</v>
+        <v>18.26666666666667</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>387.2666666666667</v>
+        <v>377.4333333333333</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>99.73999999999999</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>142.49</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>246</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2553097000000</t>
+          <t>2557400000000</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>バナナのふんわりロール２</t>
+          <t>クリーム爆盛ロールケーキ大</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>272.1333333333333</v>
+        <v>7.2</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>65.43333333333334</v>
+        <v>2.366666666666667</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>14.6</v>
+        <v>0</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>18.26666666666667</v>
+        <v>0</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>377.4333333333333</v>
+        <v>9.566666666666666</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>290.84</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>413.38</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>753</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2555045000000</t>
+          <t>2557943000000</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>全粒粉入り湯種ロール３個</t>
+          <t>ミニシューＢＯＸ</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>14.96666666666667</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>3</v>
+        <v>5.166666666666667</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>2.9</v>
+        <v>0</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>1.533333333333333</v>
+        <v>0</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>5.833333333333333</v>
+        <v>0</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>22.56666666666667</v>
+        <v>20.13333333333333</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>229.68</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>327.96</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>537</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2555056000000</t>
+          <t>2562603000000</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ふわもちホテルロール３個</t>
+          <t>お芋ムースのパンナコッタ</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>38.7</v>
+        <v>106.8666666666667</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>3.3</v>
+        <v>35.46666666666667</v>
       </c>
       <c r="E16" s="3" t="n">
+        <v>3.366666666666667</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.7333333333333333</v>
+      </c>
+      <c r="G16" s="3" t="n">
         <v>2.766666666666667</v>
       </c>
-      <c r="F16" s="3" t="n">
-        <v>1.666666666666667</v>
-      </c>
-      <c r="G16" s="3" t="n">
-        <v>5.566666666666666</v>
-      </c>
       <c r="H16" s="3" t="n">
-        <v>52</v>
+        <v>149.2</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>143.76</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>205.37</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>289</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2556874000000</t>
+          <t>2562607000000</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>塩パン２個</t>
+          <t>パキっとろっお芋ティラミス</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>26.83333333333333</v>
+        <v>100.4</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>26.5</v>
+        <v>34.43333333333333</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>3.766666666666667</v>
+        <v>3.866666666666667</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>1.1</v>
+        <v>1.833333333333333</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>2.933333333333333</v>
+        <v>3.133333333333333</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>61.13333333333333</v>
+        <v>143.6666666666667</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>127.71</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>182.13</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>289</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2557400000000</t>
+          <t>2562746000000</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>クリーム爆盛ロールケーキ大</t>
+          <t>もちっと芋の暴れん坊</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>7.2</v>
+        <v>83.66666666666667</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>2.366666666666667</v>
+        <v>34.1</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0</v>
+        <v>2.033333333333333</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>0</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>9.566666666666666</v>
+        <v>122.4333333333333</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>142.12</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>203.05</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>289</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2557943000000</t>
+          <t>2562748000000</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ミニシューＢＯＸ</t>
+          <t>素材を感じる焼き芋ロール</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>14.96666666666667</v>
+        <v>92.36666666666666</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>5.166666666666667</v>
+        <v>34.3</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>0</v>
+        <v>2.633333333333333</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>0</v>
+        <v>3.766666666666667</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>20.13333333333333</v>
+        <v>137.2666666666667</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>220.72</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>315.31</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>429</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2558109000000</t>
+          <t>2569447000000</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>チーズ塩パン２個</t>
+          <t>みかんの牛乳寒天　小</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>18.7</v>
+        <v>124.2666666666667</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>14.2</v>
+        <v>42.6</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0</v>
+        <v>10.33333333333333</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>0</v>
+        <v>9.366666666666667</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>0</v>
+        <v>9.566666666666666</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>32.9</v>
+        <v>196.1333333333333</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>89.54000000000001</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>121.63</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>181</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2562603000000</t>
+          <t>2569455000000</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>お芋ムースのパンナコッタ</t>
+          <t>みかんの牛乳寒天２</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>106.8666666666667</v>
+        <v>87.96666666666667</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>35.46666666666667</v>
+        <v>36.2</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>3.366666666666667</v>
+        <v>5.433333333333334</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0.7333333333333333</v>
+        <v>6.633333333333334</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>2.766666666666667</v>
+        <v>7.3</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>149.2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>2562607000000</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>パキっとろっお芋ティラミス</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>100.4</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>34.43333333333333</v>
-      </c>
-      <c r="E22" s="3" t="n">
-        <v>3.866666666666667</v>
-      </c>
-      <c r="F22" s="3" t="n">
-        <v>1.833333333333333</v>
-      </c>
-      <c r="G22" s="3" t="n">
-        <v>3.133333333333333</v>
-      </c>
-      <c r="H22" s="3" t="n">
-        <v>143.6666666666667</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>2562746000000</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>もちっと芋の暴れん坊</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>83.66666666666667</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>2.033333333333333</v>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>0.5333333333333333</v>
-      </c>
-      <c r="G23" s="3" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="H23" s="3" t="n">
-        <v>122.4333333333333</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>2562748000000</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>素材を感じる焼き芋ロール</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>92.36666666666666</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>34.3</v>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="F24" s="3" t="n">
-        <v>2.633333333333333</v>
-      </c>
-      <c r="G24" s="3" t="n">
-        <v>3.766666666666667</v>
-      </c>
-      <c r="H24" s="3" t="n">
-        <v>137.2666666666667</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>2569447000000</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>みかんの牛乳寒天　小</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>124.2666666666667</v>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>42.6</v>
-      </c>
-      <c r="E25" s="3" t="n">
-        <v>10.33333333333333</v>
-      </c>
-      <c r="F25" s="3" t="n">
-        <v>9.366666666666667</v>
-      </c>
-      <c r="G25" s="3" t="n">
-        <v>9.566666666666666</v>
-      </c>
-      <c r="H25" s="3" t="n">
-        <v>196.1333333333333</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>2569455000000</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>みかんの牛乳寒天２</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>87.96666666666667</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>36.2</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>5.433333333333334</v>
-      </c>
-      <c r="F26" s="3" t="n">
-        <v>6.633333333333334</v>
-      </c>
-      <c r="G26" s="3" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="H26" s="3" t="n">
         <v>143.5333333333333</v>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>2831000274577</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>南蛮（生もも）１０枚ＫＩＴ</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="3" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>2831000568690</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>たっぷりトマトピザＫＩＴ</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="n">
-        <v>6.066666666666666</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="3" t="n">
-        <v>6.066666666666666</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>2831000588360</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>照焼きチキンＫＩＴ２</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="n">
-        <v>4.533333333333333</v>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="E29" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="3" t="n">
-        <v>6.933333333333334</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>2831000599120</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>ミックスピザ４</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="n">
-        <v>26.76666666666667</v>
-      </c>
-      <c r="D30" s="3" t="n">
-        <v>7.333333333333333</v>
-      </c>
-      <c r="E30" s="3" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F30" s="3" t="n">
-        <v>0.06666666666666667</v>
-      </c>
-      <c r="G30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="3" t="n">
-        <v>35.36666666666667</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>2831000599816</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>照り焼きチキンピザＫＩＴ４</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="n">
-        <v>30.56666666666667</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>6.433333333333334</v>
-      </c>
-      <c r="E31" s="3" t="n">
-        <v>1.866666666666667</v>
-      </c>
-      <c r="F31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="3" t="n">
-        <v>38.86666666666667</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>2831000629186</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>福島生姜焼きＫＩＴ</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>4.033333333333333</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="3" t="n">
-        <v>4.933333333333334</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>2831000634500</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>豚ももスライスＫＩＴ</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>3.566666666666667</v>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="3" t="n">
-        <v>3.566666666666667</v>
+      <c r="I21" s="3" t="n">
+        <v>132.32</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>179.1</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -1452,13 +1295,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="3" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1482,6 +1327,21 @@
           <t>発注数÷30</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PC原価</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>店原価</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>店売価</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1500,6 +1360,15 @@
       <c r="D2" s="3" t="n">
         <v>304.3</v>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>110.01</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>150.7</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1518,6 +1387,15 @@
       <c r="D3" s="3" t="n">
         <v>116.2666666666667</v>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>207.92</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>284.82</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>429</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1536,6 +1414,15 @@
       <c r="D4" s="3" t="n">
         <v>134</v>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>134.34</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>184.03</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1554,6 +1441,15 @@
       <c r="D5" s="3" t="n">
         <v>44.73333333333333</v>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>166.68</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>225.55</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>375</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1572,6 +1468,15 @@
       <c r="D6" s="3" t="n">
         <v>132.9666666666667</v>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>86.09</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>117.89</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1590,6 +1495,15 @@
       <c r="D7" s="3" t="n">
         <v>446.4666666666666</v>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>94.97</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1608,6 +1522,15 @@
       <c r="D8" s="3" t="n">
         <v>75.36666666666666</v>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>130.32</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>177.54</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1626,6 +1549,15 @@
       <c r="D9" s="3" t="n">
         <v>111.2</v>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>158.83</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>217.58</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1644,6 +1576,15 @@
       <c r="D10" s="3" t="n">
         <v>494.7</v>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>100.98</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>136.14</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1662,6 +1603,15 @@
       <c r="D11" s="3" t="n">
         <v>272.7</v>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>91.98</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>125.06</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1680,6 +1630,15 @@
       <c r="D12" s="3" t="n">
         <v>142.2333333333333</v>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>88.78</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>121.62</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1698,6 +1657,15 @@
       <c r="D13" s="3" t="n">
         <v>309.7333333333333</v>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>88.66</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>134.33</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>257</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1716,6 +1684,15 @@
       <c r="D14" s="3" t="n">
         <v>272.1333333333333</v>
       </c>
+      <c r="E14" s="3" t="n">
+        <v>99.73999999999999</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>142.49</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>246</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1734,6 +1711,15 @@
       <c r="D15" s="3" t="n">
         <v>9.300000000000001</v>
       </c>
+      <c r="E15" s="3" t="n">
+        <v>45.67</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1752,6 +1738,15 @@
       <c r="D16" s="3" t="n">
         <v>38.7</v>
       </c>
+      <c r="E16" s="3" t="n">
+        <v>39.19</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>58.58</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1770,6 +1765,15 @@
       <c r="D17" s="3" t="n">
         <v>26.83333333333333</v>
       </c>
+      <c r="E17" s="3" t="n">
+        <v>55.76</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>84.45999999999999</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1788,6 +1792,15 @@
       <c r="D18" s="3" t="n">
         <v>7.2</v>
       </c>
+      <c r="E18" s="3" t="n">
+        <v>290.84</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>413.38</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>753</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1806,6 +1819,15 @@
       <c r="D19" s="3" t="n">
         <v>14.96666666666667</v>
       </c>
+      <c r="E19" s="3" t="n">
+        <v>229.68</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>327.96</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>537</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1824,6 +1846,15 @@
       <c r="D20" s="3" t="n">
         <v>18.7</v>
       </c>
+      <c r="E20" s="3" t="n">
+        <v>77.34999999999999</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>117.2</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>246</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1842,6 +1873,15 @@
       <c r="D21" s="3" t="n">
         <v>106.8666666666667</v>
       </c>
+      <c r="E21" s="3" t="n">
+        <v>143.76</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>205.37</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1860,6 +1900,15 @@
       <c r="D22" s="3" t="n">
         <v>100.4</v>
       </c>
+      <c r="E22" s="3" t="n">
+        <v>127.71</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>182.13</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1878,6 +1927,15 @@
       <c r="D23" s="3" t="n">
         <v>83.66666666666667</v>
       </c>
+      <c r="E23" s="3" t="n">
+        <v>142.12</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>203.05</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1896,6 +1954,15 @@
       <c r="D24" s="3" t="n">
         <v>92.36666666666666</v>
       </c>
+      <c r="E24" s="3" t="n">
+        <v>220.72</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>315.31</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>429</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1914,6 +1981,15 @@
       <c r="D25" s="3" t="n">
         <v>124.2666666666667</v>
       </c>
+      <c r="E25" s="3" t="n">
+        <v>89.54000000000001</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>121.63</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>181</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1932,6 +2008,15 @@
       <c r="D26" s="3" t="n">
         <v>87.96666666666667</v>
       </c>
+      <c r="E26" s="3" t="n">
+        <v>132.32</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>179.1</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>267</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1950,6 +2035,15 @@
       <c r="D27" s="3" t="n">
         <v>0.5</v>
       </c>
+      <c r="E27" s="3" t="n">
+        <v>947.6</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>1202.6</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>945</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1968,6 +2062,15 @@
       <c r="D28" s="3" t="n">
         <v>6.066666666666666</v>
       </c>
+      <c r="E28" s="3" t="n">
+        <v>173.65</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>218.65</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>235</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1986,6 +2089,15 @@
       <c r="D29" s="3" t="n">
         <v>4.533333333333333</v>
       </c>
+      <c r="E29" s="3" t="n">
+        <v>1451.69</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>1825.13</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2004,6 +2116,15 @@
       <c r="D30" s="3" t="n">
         <v>26.76666666666667</v>
       </c>
+      <c r="E30" s="3" t="n">
+        <v>190.51</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>239.21</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>258</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2022,6 +2143,15 @@
       <c r="D31" s="3" t="n">
         <v>30.56666666666667</v>
       </c>
+      <c r="E31" s="3" t="n">
+        <v>290.01</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>362.51</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>390</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2040,6 +2170,15 @@
       <c r="D32" s="3" t="n">
         <v>4.033333333333333</v>
       </c>
+      <c r="E32" s="3" t="n">
+        <v>1214.09</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>1517.46</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>1608</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2057,6 +2196,15 @@
       </c>
       <c r="D33" s="3" t="n">
         <v>3.566666666666667</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>1016.44</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>1269.79</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>1267</v>
       </c>
     </row>
   </sheetData>
@@ -2070,13 +2218,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="3" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2100,6 +2250,21 @@
           <t>発注数÷30</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PC原価</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>店原価</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>店売価</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2118,6 +2283,15 @@
       <c r="D2" s="3" t="n">
         <v>55.63333333333333</v>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>110.01</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>150.7</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2136,6 +2310,15 @@
       <c r="D3" s="3" t="n">
         <v>28.5</v>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>207.92</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>284.82</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>429</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2154,6 +2337,15 @@
       <c r="D4" s="3" t="n">
         <v>31</v>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>134.34</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>184.03</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2172,6 +2364,15 @@
       <c r="D5" s="3" t="n">
         <v>19.96666666666667</v>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>166.68</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>225.55</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>375</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2190,6 +2391,15 @@
       <c r="D6" s="3" t="n">
         <v>40.9</v>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>86.09</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>117.89</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2208,6 +2418,15 @@
       <c r="D7" s="3" t="n">
         <v>84.73333333333333</v>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>94.97</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2226,6 +2445,15 @@
       <c r="D8" s="3" t="n">
         <v>19.63333333333333</v>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>130.32</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>177.54</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2244,6 +2472,15 @@
       <c r="D9" s="3" t="n">
         <v>38.9</v>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>158.83</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>217.58</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2262,6 +2499,15 @@
       <c r="D10" s="3" t="n">
         <v>111.9666666666667</v>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>100.98</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>136.14</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2280,6 +2526,15 @@
       <c r="D11" s="3" t="n">
         <v>71.5</v>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>91.98</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>125.06</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2298,6 +2553,15 @@
       <c r="D12" s="3" t="n">
         <v>42.46666666666667</v>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>88.78</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>121.62</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2316,6 +2580,15 @@
       <c r="D13" s="3" t="n">
         <v>43.93333333333333</v>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>88.66</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>134.33</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>257</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2334,6 +2607,15 @@
       <c r="D14" s="3" t="n">
         <v>65.43333333333334</v>
       </c>
+      <c r="E14" s="3" t="n">
+        <v>99.73999999999999</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>142.49</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>246</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2352,6 +2634,15 @@
       <c r="D15" s="3" t="n">
         <v>3</v>
       </c>
+      <c r="E15" s="3" t="n">
+        <v>45.67</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2370,6 +2661,15 @@
       <c r="D16" s="3" t="n">
         <v>3.3</v>
       </c>
+      <c r="E16" s="3" t="n">
+        <v>39.19</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>58.58</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2388,6 +2688,15 @@
       <c r="D17" s="3" t="n">
         <v>26.5</v>
       </c>
+      <c r="E17" s="3" t="n">
+        <v>55.76</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>84.45999999999999</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2406,6 +2715,15 @@
       <c r="D18" s="3" t="n">
         <v>2.366666666666667</v>
       </c>
+      <c r="E18" s="3" t="n">
+        <v>290.84</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>413.38</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>753</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2424,6 +2742,15 @@
       <c r="D19" s="3" t="n">
         <v>5.166666666666667</v>
       </c>
+      <c r="E19" s="3" t="n">
+        <v>229.68</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>327.96</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>537</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2442,6 +2769,15 @@
       <c r="D20" s="3" t="n">
         <v>14.2</v>
       </c>
+      <c r="E20" s="3" t="n">
+        <v>77.34999999999999</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>117.2</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>246</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2460,6 +2796,15 @@
       <c r="D21" s="3" t="n">
         <v>35.46666666666667</v>
       </c>
+      <c r="E21" s="3" t="n">
+        <v>143.76</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>205.37</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2478,6 +2823,15 @@
       <c r="D22" s="3" t="n">
         <v>34.43333333333333</v>
       </c>
+      <c r="E22" s="3" t="n">
+        <v>127.71</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>182.13</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2496,6 +2850,15 @@
       <c r="D23" s="3" t="n">
         <v>34.1</v>
       </c>
+      <c r="E23" s="3" t="n">
+        <v>142.12</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>203.05</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2514,6 +2877,15 @@
       <c r="D24" s="3" t="n">
         <v>34.3</v>
       </c>
+      <c r="E24" s="3" t="n">
+        <v>220.72</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>315.31</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>429</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2532,6 +2904,15 @@
       <c r="D25" s="3" t="n">
         <v>42.6</v>
       </c>
+      <c r="E25" s="3" t="n">
+        <v>89.54000000000001</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>121.63</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>181</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2550,6 +2931,15 @@
       <c r="D26" s="3" t="n">
         <v>36.2</v>
       </c>
+      <c r="E26" s="3" t="n">
+        <v>132.32</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>179.1</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>267</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2568,6 +2958,15 @@
       <c r="D27" s="3" t="n">
         <v>1.9</v>
       </c>
+      <c r="E27" s="3" t="n">
+        <v>1451.69</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>1825.13</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2586,6 +2985,15 @@
       <c r="D28" s="3" t="n">
         <v>7.333333333333333</v>
       </c>
+      <c r="E28" s="3" t="n">
+        <v>190.51</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>239.21</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>258</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2604,6 +3012,15 @@
       <c r="D29" s="3" t="n">
         <v>6.433333333333334</v>
       </c>
+      <c r="E29" s="3" t="n">
+        <v>290.01</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>362.51</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>390</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2621,6 +3038,15 @@
       </c>
       <c r="D30" s="3" t="n">
         <v>0.9</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>1214.09</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>1517.46</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>1608</v>
       </c>
     </row>
   </sheetData>
@@ -2634,13 +3060,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="3" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2664,6 +3092,21 @@
           <t>発注数÷30</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PC原価</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>店原価</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>店売価</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2682,6 +3125,15 @@
       <c r="D2" s="3" t="n">
         <v>10.13333333333333</v>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>110.01</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>150.7</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2700,6 +3152,15 @@
       <c r="D3" s="3" t="n">
         <v>7.366666666666666</v>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>207.92</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>284.82</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>429</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2718,6 +3179,15 @@
       <c r="D4" s="3" t="n">
         <v>7.2</v>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>134.34</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>184.03</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2736,6 +3206,15 @@
       <c r="D5" s="3" t="n">
         <v>1.266666666666667</v>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>166.68</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>225.55</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>375</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2754,6 +3233,15 @@
       <c r="D6" s="3" t="n">
         <v>4.433333333333334</v>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>86.09</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>117.89</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2772,6 +3260,15 @@
       <c r="D7" s="3" t="n">
         <v>15.56666666666667</v>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>94.97</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2790,6 +3287,15 @@
       <c r="D8" s="3" t="n">
         <v>1.5</v>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>130.32</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>177.54</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2808,6 +3314,15 @@
       <c r="D9" s="3" t="n">
         <v>8.866666666666667</v>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>158.83</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>217.58</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2826,6 +3341,15 @@
       <c r="D10" s="3" t="n">
         <v>17.33333333333333</v>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>100.98</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>136.14</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2844,6 +3368,15 @@
       <c r="D11" s="3" t="n">
         <v>10.66666666666667</v>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>91.98</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>125.06</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2862,6 +3395,15 @@
       <c r="D12" s="3" t="n">
         <v>9.766666666666667</v>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>88.78</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>121.62</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2880,6 +3422,15 @@
       <c r="D13" s="3" t="n">
         <v>7</v>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>99.73999999999999</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>142.49</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>246</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2898,6 +3449,15 @@
       <c r="D14" s="3" t="n">
         <v>2.9</v>
       </c>
+      <c r="E14" s="3" t="n">
+        <v>45.67</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2916,6 +3476,15 @@
       <c r="D15" s="3" t="n">
         <v>2.766666666666667</v>
       </c>
+      <c r="E15" s="3" t="n">
+        <v>39.19</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>58.58</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2934,6 +3503,15 @@
       <c r="D16" s="3" t="n">
         <v>3.766666666666667</v>
       </c>
+      <c r="E16" s="3" t="n">
+        <v>55.76</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>84.45999999999999</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2952,6 +3530,15 @@
       <c r="D17" s="3" t="n">
         <v>3.366666666666667</v>
       </c>
+      <c r="E17" s="3" t="n">
+        <v>143.76</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>205.37</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2970,6 +3557,15 @@
       <c r="D18" s="3" t="n">
         <v>3.866666666666667</v>
       </c>
+      <c r="E18" s="3" t="n">
+        <v>127.71</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>182.13</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2988,6 +3584,15 @@
       <c r="D19" s="3" t="n">
         <v>2.033333333333333</v>
       </c>
+      <c r="E19" s="3" t="n">
+        <v>142.12</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>203.05</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3006,6 +3611,15 @@
       <c r="D20" s="3" t="n">
         <v>4.2</v>
       </c>
+      <c r="E20" s="3" t="n">
+        <v>220.72</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>315.31</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>429</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3024,6 +3638,15 @@
       <c r="D21" s="3" t="n">
         <v>10.33333333333333</v>
       </c>
+      <c r="E21" s="3" t="n">
+        <v>89.54000000000001</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>121.63</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>181</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3042,6 +3665,15 @@
       <c r="D22" s="3" t="n">
         <v>5.433333333333334</v>
       </c>
+      <c r="E22" s="3" t="n">
+        <v>132.32</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>179.1</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>267</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3060,6 +3692,15 @@
       <c r="D23" s="3" t="n">
         <v>0.5</v>
       </c>
+      <c r="E23" s="3" t="n">
+        <v>1451.69</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>1825.13</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3078,6 +3719,15 @@
       <c r="D24" s="3" t="n">
         <v>1.2</v>
       </c>
+      <c r="E24" s="3" t="n">
+        <v>190.51</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>239.21</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>258</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3095,6 +3745,15 @@
       </c>
       <c r="D25" s="3" t="n">
         <v>1.866666666666667</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>290.01</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>362.51</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>390</v>
       </c>
     </row>
   </sheetData>
@@ -3108,13 +3767,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="3" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3138,6 +3799,21 @@
           <t>発注数÷30</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PC原価</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>店原価</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>店売価</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3156,6 +3832,15 @@
       <c r="D2" s="3" t="n">
         <v>7.766666666666667</v>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>110.01</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>150.7</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3174,6 +3859,15 @@
       <c r="D3" s="3" t="n">
         <v>1.333333333333333</v>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>134.34</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>184.03</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3192,6 +3886,15 @@
       <c r="D4" s="3" t="n">
         <v>0.7</v>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>166.68</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>225.55</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>375</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3210,6 +3913,15 @@
       <c r="D5" s="3" t="n">
         <v>4.1</v>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>86.09</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>117.89</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3228,6 +3940,15 @@
       <c r="D6" s="3" t="n">
         <v>18.13333333333333</v>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>94.97</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3246,6 +3967,15 @@
       <c r="D7" s="3" t="n">
         <v>0.4333333333333333</v>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>130.32</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>177.54</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3264,6 +3994,15 @@
       <c r="D8" s="3" t="n">
         <v>5.366666666666666</v>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>158.83</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>217.58</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3282,6 +4021,15 @@
       <c r="D9" s="3" t="n">
         <v>17.03333333333333</v>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>100.98</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>136.14</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3300,6 +4048,15 @@
       <c r="D10" s="3" t="n">
         <v>12.93333333333333</v>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>91.98</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>125.06</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3318,6 +4075,15 @@
       <c r="D11" s="3" t="n">
         <v>8.9</v>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>88.78</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>121.62</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3336,6 +4102,15 @@
       <c r="D12" s="3" t="n">
         <v>6.7</v>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>88.66</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>134.33</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>257</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3354,6 +4129,15 @@
       <c r="D13" s="3" t="n">
         <v>14.6</v>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>99.73999999999999</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>142.49</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>246</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3372,6 +4156,15 @@
       <c r="D14" s="3" t="n">
         <v>1.533333333333333</v>
       </c>
+      <c r="E14" s="3" t="n">
+        <v>45.67</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3390,6 +4183,15 @@
       <c r="D15" s="3" t="n">
         <v>1.666666666666667</v>
       </c>
+      <c r="E15" s="3" t="n">
+        <v>39.19</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>58.58</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3408,6 +4210,15 @@
       <c r="D16" s="3" t="n">
         <v>1.1</v>
       </c>
+      <c r="E16" s="3" t="n">
+        <v>55.76</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>84.45999999999999</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3426,6 +4237,15 @@
       <c r="D17" s="3" t="n">
         <v>0.7333333333333333</v>
       </c>
+      <c r="E17" s="3" t="n">
+        <v>143.76</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>205.37</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3444,6 +4264,15 @@
       <c r="D18" s="3" t="n">
         <v>1.833333333333333</v>
       </c>
+      <c r="E18" s="3" t="n">
+        <v>127.71</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>182.13</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3462,6 +4291,15 @@
       <c r="D19" s="3" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="E19" s="3" t="n">
+        <v>142.12</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>203.05</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3480,6 +4318,15 @@
       <c r="D20" s="3" t="n">
         <v>2.633333333333333</v>
       </c>
+      <c r="E20" s="3" t="n">
+        <v>220.72</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>315.31</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>429</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3498,6 +4345,15 @@
       <c r="D21" s="3" t="n">
         <v>9.366666666666667</v>
       </c>
+      <c r="E21" s="3" t="n">
+        <v>89.54000000000001</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>121.63</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>181</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3516,6 +4372,15 @@
       <c r="D22" s="3" t="n">
         <v>6.633333333333334</v>
       </c>
+      <c r="E22" s="3" t="n">
+        <v>132.32</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>179.1</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>267</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3533,6 +4398,15 @@
       </c>
       <c r="D23" s="3" t="n">
         <v>0.06666666666666667</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>190.51</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>239.21</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -3546,13 +4420,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="3" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3576,6 +4452,21 @@
           <t>発注数÷30</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PC原価</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>店原価</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>店売価</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3594,6 +4485,15 @@
       <c r="D2" s="3" t="n">
         <v>6.2</v>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>110.01</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>150.7</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3612,6 +4512,15 @@
       <c r="D3" s="3" t="n">
         <v>0.1333333333333333</v>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>207.92</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>284.82</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>429</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3630,6 +4539,15 @@
       <c r="D4" s="3" t="n">
         <v>1.5</v>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>134.34</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>184.03</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3648,6 +4566,15 @@
       <c r="D5" s="3" t="n">
         <v>1.2</v>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>166.68</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>225.55</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>375</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3666,6 +4593,15 @@
       <c r="D6" s="3" t="n">
         <v>6.966666666666667</v>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>86.09</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>117.89</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3684,6 +4620,15 @@
       <c r="D7" s="3" t="n">
         <v>23.46666666666667</v>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>69.92</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>94.97</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3702,6 +4647,15 @@
       <c r="D8" s="3" t="n">
         <v>0.6666666666666666</v>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>130.32</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>177.54</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3720,6 +4674,15 @@
       <c r="D9" s="3" t="n">
         <v>7.2</v>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>158.83</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>217.58</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3738,6 +4701,15 @@
       <c r="D10" s="3" t="n">
         <v>23.36666666666667</v>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>100.98</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>136.14</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3756,6 +4728,15 @@
       <c r="D11" s="3" t="n">
         <v>16.56666666666667</v>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>91.98</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>125.06</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3774,6 +4755,15 @@
       <c r="D12" s="3" t="n">
         <v>7.966666666666667</v>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>88.78</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>121.62</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3792,6 +4782,15 @@
       <c r="D13" s="3" t="n">
         <v>26.9</v>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>88.66</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>134.33</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>257</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3810,6 +4809,15 @@
       <c r="D14" s="3" t="n">
         <v>18.26666666666667</v>
       </c>
+      <c r="E14" s="3" t="n">
+        <v>99.73999999999999</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>142.49</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>246</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3828,6 +4836,15 @@
       <c r="D15" s="3" t="n">
         <v>5.833333333333333</v>
       </c>
+      <c r="E15" s="3" t="n">
+        <v>45.67</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3846,6 +4863,15 @@
       <c r="D16" s="3" t="n">
         <v>5.566666666666666</v>
       </c>
+      <c r="E16" s="3" t="n">
+        <v>39.19</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>58.58</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3864,6 +4890,15 @@
       <c r="D17" s="3" t="n">
         <v>2.933333333333333</v>
       </c>
+      <c r="E17" s="3" t="n">
+        <v>55.76</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>84.45999999999999</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>213</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3882,6 +4917,15 @@
       <c r="D18" s="3" t="n">
         <v>2.766666666666667</v>
       </c>
+      <c r="E18" s="3" t="n">
+        <v>143.76</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>205.37</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3900,6 +4944,15 @@
       <c r="D19" s="3" t="n">
         <v>3.133333333333333</v>
       </c>
+      <c r="E19" s="3" t="n">
+        <v>127.71</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>182.13</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3918,6 +4971,15 @@
       <c r="D20" s="3" t="n">
         <v>2.1</v>
       </c>
+      <c r="E20" s="3" t="n">
+        <v>142.12</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>203.05</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>289</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3936,6 +4998,15 @@
       <c r="D21" s="3" t="n">
         <v>3.766666666666667</v>
       </c>
+      <c r="E21" s="3" t="n">
+        <v>220.72</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>315.31</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>429</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3954,6 +5025,15 @@
       <c r="D22" s="3" t="n">
         <v>9.566666666666666</v>
       </c>
+      <c r="E22" s="3" t="n">
+        <v>89.54000000000001</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>121.63</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>181</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3971,6 +5051,15 @@
       </c>
       <c r="D23" s="3" t="n">
         <v>7.3</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>132.32</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>179.1</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -3985,7 +5074,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>